<commit_message>
add script para eliminar duplicidades
</commit_message>
<xml_diff>
--- a/output_data_cnae/output_data_cnae_full_erros.xlsx
+++ b/output_data_cnae/output_data_cnae_full_erros.xlsx
@@ -354,7 +354,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -394,42 +394,6 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F16" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>